<commit_message>
docs(gantt): revise Agile Data Science project schedule
</commit_message>
<xml_diff>
--- a/output/gantt-chart-revised/ResBack Gantt Chart Agile Data Science 2.0.xlsx
+++ b/output/gantt-chart-revised/ResBack Gantt Chart Agile Data Science 2.0.xlsx
@@ -148,7 +148,7 @@
     <t>Create interface wireframes</t>
   </si>
   <si>
-    <t>UI/UX Dev (Quina)</t>
+    <t>UI/UX Dev (Queypo)</t>
   </si>
   <si>
     <t>Interface wireframes</t>
@@ -292,7 +292,7 @@
     <t>Conduct user acceptance testing and stakeholder review</t>
   </si>
   <si>
-    <t>QA Tester (Ballesteros)</t>
+    <t>QA Tester (Viloria)</t>
   </si>
   <si>
     <t>UAT results and review findings</t>
@@ -426,7 +426,7 @@
       <name val="Arial"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -451,6 +451,12 @@
         <bgColor rgb="FF92D050"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor theme="0"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="19">
     <border/>
@@ -683,7 +689,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="39">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -748,6 +754,9 @@
     </xf>
     <xf borderId="13" fillId="2" fontId="8" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="14" fillId="5" fontId="3" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="13" fillId="2" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
     <xf borderId="14" fillId="2" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
@@ -2014,7 +2023,7 @@
       <c r="C19" s="21" t="s">
         <v>44</v>
       </c>
-      <c r="D19" s="22" t="s">
+      <c r="D19" s="27" t="s">
         <v>45</v>
       </c>
       <c r="E19" s="23">
@@ -2160,7 +2169,7 @@
       <c r="C21" s="21" t="s">
         <v>49</v>
       </c>
-      <c r="D21" s="22" t="s">
+      <c r="D21" s="27" t="s">
         <v>45</v>
       </c>
       <c r="E21" s="23">
@@ -2229,26 +2238,26 @@
       </c>
     </row>
     <row r="22" ht="14.25" customHeight="1">
-      <c r="B22" s="27"/>
-      <c r="C22" s="28"/>
-      <c r="D22" s="28"/>
-      <c r="E22" s="28"/>
-      <c r="F22" s="28"/>
-      <c r="G22" s="28"/>
-      <c r="H22" s="28"/>
-      <c r="I22" s="28"/>
-      <c r="J22" s="28"/>
-      <c r="K22" s="28"/>
-      <c r="L22" s="28"/>
-      <c r="M22" s="28"/>
-      <c r="N22" s="28"/>
-      <c r="O22" s="28"/>
-      <c r="P22" s="28"/>
-      <c r="Q22" s="28"/>
-      <c r="R22" s="28"/>
-      <c r="S22" s="28"/>
-      <c r="T22" s="28"/>
-      <c r="U22" s="29"/>
+      <c r="B22" s="28"/>
+      <c r="C22" s="29"/>
+      <c r="D22" s="29"/>
+      <c r="E22" s="29"/>
+      <c r="F22" s="29"/>
+      <c r="G22" s="29"/>
+      <c r="H22" s="29"/>
+      <c r="I22" s="29"/>
+      <c r="J22" s="29"/>
+      <c r="K22" s="29"/>
+      <c r="L22" s="29"/>
+      <c r="M22" s="29"/>
+      <c r="N22" s="29"/>
+      <c r="O22" s="29"/>
+      <c r="P22" s="29"/>
+      <c r="Q22" s="29"/>
+      <c r="R22" s="29"/>
+      <c r="S22" s="29"/>
+      <c r="T22" s="29"/>
+      <c r="U22" s="30"/>
     </row>
     <row r="23" ht="14.25" customHeight="1">
       <c r="B23" s="20" t="s">
@@ -2695,7 +2704,7 @@
       <c r="C29" s="21" t="s">
         <v>64</v>
       </c>
-      <c r="D29" s="22" t="s">
+      <c r="D29" s="27" t="s">
         <v>45</v>
       </c>
       <c r="E29" s="23">
@@ -2983,26 +2992,26 @@
       </c>
     </row>
     <row r="33" ht="14.25" customHeight="1">
-      <c r="B33" s="27"/>
-      <c r="C33" s="28"/>
-      <c r="D33" s="28"/>
-      <c r="E33" s="28"/>
-      <c r="F33" s="28"/>
-      <c r="G33" s="28"/>
-      <c r="H33" s="28"/>
-      <c r="I33" s="28"/>
-      <c r="J33" s="28"/>
-      <c r="K33" s="28"/>
-      <c r="L33" s="28"/>
-      <c r="M33" s="28"/>
-      <c r="N33" s="28"/>
-      <c r="O33" s="28"/>
-      <c r="P33" s="28"/>
-      <c r="Q33" s="28"/>
-      <c r="R33" s="28"/>
-      <c r="S33" s="28"/>
-      <c r="T33" s="28"/>
-      <c r="U33" s="29"/>
+      <c r="B33" s="28"/>
+      <c r="C33" s="29"/>
+      <c r="D33" s="29"/>
+      <c r="E33" s="29"/>
+      <c r="F33" s="29"/>
+      <c r="G33" s="29"/>
+      <c r="H33" s="29"/>
+      <c r="I33" s="29"/>
+      <c r="J33" s="29"/>
+      <c r="K33" s="29"/>
+      <c r="L33" s="29"/>
+      <c r="M33" s="29"/>
+      <c r="N33" s="29"/>
+      <c r="O33" s="29"/>
+      <c r="P33" s="29"/>
+      <c r="Q33" s="29"/>
+      <c r="R33" s="29"/>
+      <c r="S33" s="29"/>
+      <c r="T33" s="29"/>
+      <c r="U33" s="30"/>
     </row>
     <row r="34" ht="14.25" customHeight="1">
       <c r="B34" s="20" t="s">
@@ -3011,7 +3020,7 @@
       <c r="C34" s="21" t="s">
         <v>73</v>
       </c>
-      <c r="D34" s="22" t="s">
+      <c r="D34" s="27" t="s">
         <v>45</v>
       </c>
       <c r="E34" s="23">
@@ -3084,7 +3093,7 @@
       <c r="C35" s="21" t="s">
         <v>75</v>
       </c>
-      <c r="D35" s="22" t="s">
+      <c r="D35" s="27" t="s">
         <v>45</v>
       </c>
       <c r="E35" s="23">
@@ -3153,26 +3162,26 @@
       </c>
     </row>
     <row r="36" ht="14.25" customHeight="1">
-      <c r="B36" s="27"/>
-      <c r="C36" s="28"/>
-      <c r="D36" s="28"/>
-      <c r="E36" s="28"/>
-      <c r="F36" s="28"/>
-      <c r="G36" s="28"/>
-      <c r="H36" s="28"/>
-      <c r="I36" s="28"/>
-      <c r="J36" s="28"/>
-      <c r="K36" s="28"/>
-      <c r="L36" s="28"/>
-      <c r="M36" s="28"/>
-      <c r="N36" s="28"/>
-      <c r="O36" s="28"/>
-      <c r="P36" s="28"/>
-      <c r="Q36" s="28"/>
-      <c r="R36" s="28"/>
-      <c r="S36" s="28"/>
-      <c r="T36" s="28"/>
-      <c r="U36" s="29"/>
+      <c r="B36" s="28"/>
+      <c r="C36" s="29"/>
+      <c r="D36" s="29"/>
+      <c r="E36" s="29"/>
+      <c r="F36" s="29"/>
+      <c r="G36" s="29"/>
+      <c r="H36" s="29"/>
+      <c r="I36" s="29"/>
+      <c r="J36" s="29"/>
+      <c r="K36" s="29"/>
+      <c r="L36" s="29"/>
+      <c r="M36" s="29"/>
+      <c r="N36" s="29"/>
+      <c r="O36" s="29"/>
+      <c r="P36" s="29"/>
+      <c r="Q36" s="29"/>
+      <c r="R36" s="29"/>
+      <c r="S36" s="29"/>
+      <c r="T36" s="29"/>
+      <c r="U36" s="30"/>
     </row>
     <row r="37" ht="14.25" customHeight="1">
       <c r="B37" s="20" t="s">
@@ -3323,26 +3332,26 @@
       </c>
     </row>
     <row r="39" ht="14.25" customHeight="1">
-      <c r="B39" s="27"/>
-      <c r="C39" s="28"/>
-      <c r="D39" s="28"/>
-      <c r="E39" s="28"/>
-      <c r="F39" s="28"/>
-      <c r="G39" s="28"/>
-      <c r="H39" s="28"/>
-      <c r="I39" s="28"/>
-      <c r="J39" s="28"/>
-      <c r="K39" s="28"/>
-      <c r="L39" s="28"/>
-      <c r="M39" s="28"/>
-      <c r="N39" s="28"/>
-      <c r="O39" s="28"/>
-      <c r="P39" s="28"/>
-      <c r="Q39" s="28"/>
-      <c r="R39" s="28"/>
-      <c r="S39" s="28"/>
-      <c r="T39" s="28"/>
-      <c r="U39" s="29"/>
+      <c r="B39" s="28"/>
+      <c r="C39" s="29"/>
+      <c r="D39" s="29"/>
+      <c r="E39" s="29"/>
+      <c r="F39" s="29"/>
+      <c r="G39" s="29"/>
+      <c r="H39" s="29"/>
+      <c r="I39" s="29"/>
+      <c r="J39" s="29"/>
+      <c r="K39" s="29"/>
+      <c r="L39" s="29"/>
+      <c r="M39" s="29"/>
+      <c r="N39" s="29"/>
+      <c r="O39" s="29"/>
+      <c r="P39" s="29"/>
+      <c r="Q39" s="29"/>
+      <c r="R39" s="29"/>
+      <c r="S39" s="29"/>
+      <c r="T39" s="29"/>
+      <c r="U39" s="30"/>
     </row>
     <row r="40" ht="14.25" customHeight="1">
       <c r="B40" s="20" t="s">
@@ -3570,7 +3579,7 @@
       <c r="C43" s="21" t="s">
         <v>89</v>
       </c>
-      <c r="D43" s="22" t="s">
+      <c r="D43" s="27" t="s">
         <v>45</v>
       </c>
       <c r="E43" s="23">
@@ -3639,26 +3648,26 @@
       </c>
     </row>
     <row r="44" ht="14.25" customHeight="1">
-      <c r="B44" s="27"/>
-      <c r="C44" s="28"/>
-      <c r="D44" s="28"/>
-      <c r="E44" s="28"/>
-      <c r="F44" s="28"/>
-      <c r="G44" s="28"/>
-      <c r="H44" s="28"/>
-      <c r="I44" s="28"/>
-      <c r="J44" s="28"/>
-      <c r="K44" s="28"/>
-      <c r="L44" s="28"/>
-      <c r="M44" s="28"/>
-      <c r="N44" s="28"/>
-      <c r="O44" s="28"/>
-      <c r="P44" s="28"/>
-      <c r="Q44" s="28"/>
-      <c r="R44" s="28"/>
-      <c r="S44" s="28"/>
-      <c r="T44" s="28"/>
-      <c r="U44" s="29"/>
+      <c r="B44" s="28"/>
+      <c r="C44" s="29"/>
+      <c r="D44" s="29"/>
+      <c r="E44" s="29"/>
+      <c r="F44" s="29"/>
+      <c r="G44" s="29"/>
+      <c r="H44" s="29"/>
+      <c r="I44" s="29"/>
+      <c r="J44" s="29"/>
+      <c r="K44" s="29"/>
+      <c r="L44" s="29"/>
+      <c r="M44" s="29"/>
+      <c r="N44" s="29"/>
+      <c r="O44" s="29"/>
+      <c r="P44" s="29"/>
+      <c r="Q44" s="29"/>
+      <c r="R44" s="29"/>
+      <c r="S44" s="29"/>
+      <c r="T44" s="29"/>
+      <c r="U44" s="30"/>
     </row>
     <row r="45" ht="14.25" customHeight="1">
       <c r="B45" s="20" t="s">
@@ -3667,7 +3676,7 @@
       <c r="C45" s="21" t="s">
         <v>92</v>
       </c>
-      <c r="D45" s="22" t="s">
+      <c r="D45" s="27" t="s">
         <v>93</v>
       </c>
       <c r="E45" s="23">
@@ -3809,26 +3818,26 @@
       </c>
     </row>
     <row r="47" ht="14.25" customHeight="1">
-      <c r="B47" s="27"/>
-      <c r="C47" s="28"/>
-      <c r="D47" s="28"/>
-      <c r="E47" s="28"/>
-      <c r="F47" s="28"/>
-      <c r="G47" s="28"/>
-      <c r="H47" s="28"/>
-      <c r="I47" s="28"/>
-      <c r="J47" s="28"/>
-      <c r="K47" s="28"/>
-      <c r="L47" s="28"/>
-      <c r="M47" s="28"/>
-      <c r="N47" s="28"/>
-      <c r="O47" s="28"/>
-      <c r="P47" s="28"/>
-      <c r="Q47" s="28"/>
-      <c r="R47" s="28"/>
-      <c r="S47" s="28"/>
-      <c r="T47" s="28"/>
-      <c r="U47" s="29"/>
+      <c r="B47" s="28"/>
+      <c r="C47" s="29"/>
+      <c r="D47" s="29"/>
+      <c r="E47" s="29"/>
+      <c r="F47" s="29"/>
+      <c r="G47" s="29"/>
+      <c r="H47" s="29"/>
+      <c r="I47" s="29"/>
+      <c r="J47" s="29"/>
+      <c r="K47" s="29"/>
+      <c r="L47" s="29"/>
+      <c r="M47" s="29"/>
+      <c r="N47" s="29"/>
+      <c r="O47" s="29"/>
+      <c r="P47" s="29"/>
+      <c r="Q47" s="29"/>
+      <c r="R47" s="29"/>
+      <c r="S47" s="29"/>
+      <c r="T47" s="29"/>
+      <c r="U47" s="30"/>
     </row>
     <row r="48" ht="14.25" customHeight="1">
       <c r="B48" s="20" t="s">
@@ -3910,7 +3919,7 @@
       <c r="C49" s="21" t="s">
         <v>100</v>
       </c>
-      <c r="D49" s="22" t="s">
+      <c r="D49" s="27" t="s">
         <v>93</v>
       </c>
       <c r="E49" s="23">
@@ -4056,7 +4065,7 @@
       <c r="C51" s="21" t="s">
         <v>104</v>
       </c>
-      <c r="D51" s="22" t="s">
+      <c r="D51" s="27" t="s">
         <v>93</v>
       </c>
       <c r="E51" s="23">
@@ -4129,7 +4138,7 @@
       <c r="C52" s="21" t="s">
         <v>106</v>
       </c>
-      <c r="D52" s="22" t="s">
+      <c r="D52" s="27" t="s">
         <v>93</v>
       </c>
       <c r="E52" s="23">
@@ -4198,26 +4207,26 @@
       </c>
     </row>
     <row r="53" ht="14.25" customHeight="1">
-      <c r="B53" s="27"/>
-      <c r="C53" s="28"/>
-      <c r="D53" s="28"/>
-      <c r="E53" s="28"/>
-      <c r="F53" s="28"/>
-      <c r="G53" s="28"/>
-      <c r="H53" s="28"/>
-      <c r="I53" s="28"/>
-      <c r="J53" s="28"/>
-      <c r="K53" s="28"/>
-      <c r="L53" s="28"/>
-      <c r="M53" s="28"/>
-      <c r="N53" s="28"/>
-      <c r="O53" s="28"/>
-      <c r="P53" s="28"/>
-      <c r="Q53" s="28"/>
-      <c r="R53" s="28"/>
-      <c r="S53" s="28"/>
-      <c r="T53" s="28"/>
-      <c r="U53" s="29"/>
+      <c r="B53" s="28"/>
+      <c r="C53" s="29"/>
+      <c r="D53" s="29"/>
+      <c r="E53" s="29"/>
+      <c r="F53" s="29"/>
+      <c r="G53" s="29"/>
+      <c r="H53" s="29"/>
+      <c r="I53" s="29"/>
+      <c r="J53" s="29"/>
+      <c r="K53" s="29"/>
+      <c r="L53" s="29"/>
+      <c r="M53" s="29"/>
+      <c r="N53" s="29"/>
+      <c r="O53" s="29"/>
+      <c r="P53" s="29"/>
+      <c r="Q53" s="29"/>
+      <c r="R53" s="29"/>
+      <c r="S53" s="29"/>
+      <c r="T53" s="29"/>
+      <c r="U53" s="30"/>
     </row>
     <row r="54" ht="14.25" customHeight="1">
       <c r="B54" s="20" t="s">
@@ -4299,7 +4308,7 @@
       <c r="C55" s="21" t="s">
         <v>111</v>
       </c>
-      <c r="D55" s="22" t="s">
+      <c r="D55" s="27" t="s">
         <v>45</v>
       </c>
       <c r="E55" s="23">
@@ -4441,75 +4450,75 @@
       </c>
     </row>
     <row r="57" ht="14.25" customHeight="1">
-      <c r="B57" s="30"/>
-      <c r="C57" s="31" t="s">
+      <c r="B57" s="31"/>
+      <c r="C57" s="32" t="s">
         <v>115</v>
       </c>
-      <c r="D57" s="32" t="s">
+      <c r="D57" s="33" t="s">
         <v>20</v>
       </c>
-      <c r="E57" s="33">
+      <c r="E57" s="34">
         <v>46324.0</v>
       </c>
-      <c r="F57" s="33">
+      <c r="F57" s="34">
         <v>46326.0</v>
       </c>
-      <c r="G57" s="32" t="s">
+      <c r="G57" s="33" t="s">
         <v>17</v>
       </c>
-      <c r="H57" s="34">
+      <c r="H57" s="35">
         <f t="shared" ref="H57:T57" si="43">IF(AND(ISNUMBER($E57),ISNUMBER($F57),$E57&lt;=$F57,$E57&lt;=MIN(DATE(2026,8,3)+H$7*7-1,DATE(2026,10,31)),$F57&gt;=DATE(2026,8,3)+(H$7-1)*7),1,0)</f>
         <v>0</v>
       </c>
-      <c r="I57" s="34">
+      <c r="I57" s="35">
         <f t="shared" si="43"/>
         <v>0</v>
       </c>
-      <c r="J57" s="34">
+      <c r="J57" s="35">
         <f t="shared" si="43"/>
         <v>0</v>
       </c>
-      <c r="K57" s="34">
+      <c r="K57" s="35">
         <f t="shared" si="43"/>
         <v>0</v>
       </c>
-      <c r="L57" s="34">
+      <c r="L57" s="35">
         <f t="shared" si="43"/>
         <v>0</v>
       </c>
-      <c r="M57" s="34">
+      <c r="M57" s="35">
         <f t="shared" si="43"/>
         <v>0</v>
       </c>
-      <c r="N57" s="34">
+      <c r="N57" s="35">
         <f t="shared" si="43"/>
         <v>0</v>
       </c>
-      <c r="O57" s="34">
+      <c r="O57" s="35">
         <f t="shared" si="43"/>
         <v>0</v>
       </c>
-      <c r="P57" s="34">
+      <c r="P57" s="35">
         <f t="shared" si="43"/>
         <v>0</v>
       </c>
-      <c r="Q57" s="34">
+      <c r="Q57" s="35">
         <f t="shared" si="43"/>
         <v>0</v>
       </c>
-      <c r="R57" s="34">
+      <c r="R57" s="35">
         <f t="shared" si="43"/>
         <v>0</v>
       </c>
-      <c r="S57" s="34">
+      <c r="S57" s="35">
         <f t="shared" si="43"/>
         <v>0</v>
       </c>
-      <c r="T57" s="34">
+      <c r="T57" s="35">
         <f t="shared" si="43"/>
         <v>1</v>
       </c>
-      <c r="U57" s="35" t="s">
+      <c r="U57" s="36" t="s">
         <v>116</v>
       </c>
     </row>
@@ -4602,26 +4611,26 @@
       <c r="U61" s="2"/>
     </row>
     <row r="62" ht="33.75" customHeight="1">
-      <c r="B62" s="36"/>
-      <c r="C62" s="36"/>
-      <c r="D62" s="36"/>
-      <c r="E62" s="36"/>
-      <c r="F62" s="36"/>
-      <c r="G62" s="36"/>
-      <c r="H62" s="36"/>
-      <c r="I62" s="37"/>
-      <c r="J62" s="37"/>
-      <c r="K62" s="37"/>
-      <c r="L62" s="37"/>
-      <c r="M62" s="37"/>
-      <c r="N62" s="37"/>
-      <c r="O62" s="37"/>
-      <c r="P62" s="37"/>
-      <c r="Q62" s="37"/>
-      <c r="R62" s="37"/>
-      <c r="S62" s="37"/>
-      <c r="T62" s="37"/>
-      <c r="U62" s="37"/>
+      <c r="B62" s="37"/>
+      <c r="C62" s="37"/>
+      <c r="D62" s="37"/>
+      <c r="E62" s="37"/>
+      <c r="F62" s="37"/>
+      <c r="G62" s="37"/>
+      <c r="H62" s="37"/>
+      <c r="I62" s="38"/>
+      <c r="J62" s="38"/>
+      <c r="K62" s="38"/>
+      <c r="L62" s="38"/>
+      <c r="M62" s="38"/>
+      <c r="N62" s="38"/>
+      <c r="O62" s="38"/>
+      <c r="P62" s="38"/>
+      <c r="Q62" s="38"/>
+      <c r="R62" s="38"/>
+      <c r="S62" s="38"/>
+      <c r="T62" s="38"/>
+      <c r="U62" s="38"/>
     </row>
     <row r="63" ht="15.75" customHeight="1"/>
     <row r="64" ht="15.75" customHeight="1"/>

</xml_diff>